<commit_message>
feat(ma): add negotiation workspace + IM chart engine improvements
- deal-mgmt: contract negotiation workspace models/schemas/routers
- deal-mgmt: migration 030 for negotiation workspace tables
- frontend: negotiation issue hooks, types, workspace page updates
- im: PPTX native chart engine + section renderer chart integration
- fdd: sample workpaper updates
- docs: VDR Azure Blob Storage deployment guide

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fdd/fdd sample/Project striker_WP_취합.xlsx
+++ b/fdd/fdd sample/Project striker_WP_취합.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onedrive-global.kpmg.com/personal/hoh2_kr_kpmg_com/Documents/YTK/M&amp;A/매수자문/Project Vision- 실사/5. Report&amp;Model(DD, Val)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c31fecfadb131e8b/Documents/Coding/AMIC x PETRA Platform/fdd/fdd sample/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{89E0678A-14CC-4088-AA23-B245564F1F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="1000" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="1000" firstSheet="3" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ES &gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;" sheetId="1" r:id="rId1"/>
@@ -20975,7 +20975,7 @@
                     <a:fld id="{DBCA8C7B-519D-4AE5-9526-4D07014AFB59}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -21010,9 +21010,9 @@
                     <a:fld id="{E7B5CF5D-FCAF-4C40-A073-4C1A7D589624}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
-                    <a:endParaRPr/>
+                    <a:endParaRPr lang="ko-KR" altLang="en-US"/>
                   </a:p>
                 </c:rich>
               </c:tx>
@@ -21046,7 +21046,7 @@
                     <a:fld id="{3C9DAD3C-92F5-4C92-9FC1-2CE105A0F4E1}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -21081,9 +21081,9 @@
                     <a:fld id="{101EEC8E-29E8-47D1-AE5B-257C9646E352}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
-                    <a:endParaRPr/>
+                    <a:endParaRPr lang="ko-KR" altLang="en-US"/>
                   </a:p>
                 </c:rich>
               </c:tx>
@@ -21117,7 +21117,7 @@
                     <a:fld id="{A7D3259D-5EF8-4CDF-A997-10B3B0014832}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -21156,7 +21156,7 @@
                     <a:fld id="{A39522B2-F638-4AEB-8B1C-DA574FF88324}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -23269,7 +23269,7 @@
                     <a:fld id="{E7B5CF5D-FCAF-4C40-A073-4C1A7D589624}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -23308,7 +23308,7 @@
                     <a:fld id="{3C9DAD3C-92F5-4C92-9FC1-2CE105A0F4E1}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -23347,7 +23347,7 @@
                     <a:fld id="{101EEC8E-29E8-47D1-AE5B-257C9646E352}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -23386,7 +23386,7 @@
                     <a:fld id="{A39522B2-F638-4AEB-8B1C-DA574FF88324}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -25450,7 +25450,7 @@
                     <a:fld id="{E7B5CF5D-FCAF-4C40-A073-4C1A7D589624}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -25489,7 +25489,7 @@
                     <a:fld id="{3C9DAD3C-92F5-4C92-9FC1-2CE105A0F4E1}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -25528,7 +25528,7 @@
                     <a:fld id="{101EEC8E-29E8-47D1-AE5B-257C9646E352}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -25567,7 +25567,7 @@
                     <a:fld id="{A39522B2-F638-4AEB-8B1C-DA574FF88324}" type="VALUE">
                       <a:rPr lang="en-US" altLang="ko-KR"/>
                       <a:pPr/>
-                      <a:t>[]</a:t>
+                      <a:t>[값]</a:t>
                     </a:fld>
                     <a:r>
                       <a:rPr lang="en-US" altLang="ko-KR"/>
@@ -27633,7 +27633,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$1:$C$11" spid="_x0000_s20542"/>
+                  <a14:cameraTool cellRange="$B$1:$C$11" spid="_x0000_s20546"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -27680,7 +27680,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>10</xdr:col>
-          <xdr:colOff>571500</xdr:colOff>
+          <xdr:colOff>600075</xdr:colOff>
           <xdr:row>29</xdr:row>
           <xdr:rowOff>76200</xdr:rowOff>
         </xdr:to>
@@ -27697,7 +27697,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$F$13:$G$26" spid="_x0000_s20543"/>
+                  <a14:cameraTool cellRange="$F$13:$G$26" spid="_x0000_s20547"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -27711,8 +27711,8 @@
           </xdr:blipFill>
           <xdr:spPr bwMode="auto">
             <a:xfrm>
-              <a:off x="9725025" y="2609850"/>
-              <a:ext cx="3600450" cy="2390775"/>
+              <a:off x="9642475" y="2609850"/>
+              <a:ext cx="3600450" cy="2387600"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -27946,7 +27946,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$1:$E$34" spid="_x0000_s8325"/>
+                  <a14:cameraTool cellRange="$A$1:$E$34" spid="_x0000_s8333"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28010,7 +28010,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$40:$E$49" spid="_x0000_s8326"/>
+                  <a14:cameraTool cellRange="$A$40:$E$49" spid="_x0000_s8334"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28074,7 +28074,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$59:$E$65" spid="_x0000_s8327"/>
+                  <a14:cameraTool cellRange="$A$59:$E$65" spid="_x0000_s8335"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28138,7 +28138,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$52:$E$57" spid="_x0000_s8328"/>
+                  <a14:cameraTool cellRange="$A$52:$E$57" spid="_x0000_s8336"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28283,7 +28283,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$2:$H$15" spid="_x0000_s16416"/>
+                  <a14:cameraTool cellRange="$B$2:$H$15" spid="_x0000_s16418"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28510,7 +28510,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$2:$F$16" spid="_x0000_s49167"/>
+                  <a14:cameraTool cellRange="$B$2:$F$16" spid="_x0000_s49171"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28574,7 +28574,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$18:$F$31" spid="_x0000_s49168"/>
+                  <a14:cameraTool cellRange="$B$18:$F$31" spid="_x0000_s49172"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28763,7 +28763,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$2:$F$7" spid="_x0000_s15423"/>
+                  <a14:cameraTool cellRange="$B$2:$F$7" spid="_x0000_s15427"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28827,7 +28827,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$9:$F$23" spid="_x0000_s15424"/>
+                  <a14:cameraTool cellRange="$B$9:$F$23" spid="_x0000_s15428"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28896,7 +28896,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$1:$G$8" spid="_x0000_s18456"/>
+                  <a14:cameraTool cellRange="$A$1:$G$8" spid="_x0000_s18458"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -28965,7 +28965,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$1:$E$34" spid="_x0000_s21617"/>
+                  <a14:cameraTool cellRange="$A$1:$E$34" spid="_x0000_s21625"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29029,7 +29029,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$40:$E$49" spid="_x0000_s21618"/>
+                  <a14:cameraTool cellRange="$A$40:$E$49" spid="_x0000_s21626"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29093,7 +29093,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$59:$E$65" spid="_x0000_s21619"/>
+                  <a14:cameraTool cellRange="$A$59:$E$65" spid="_x0000_s21627"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29157,7 +29157,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$52:$E$57" spid="_x0000_s21620"/>
+                  <a14:cameraTool cellRange="$A$52:$E$57" spid="_x0000_s21628"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29338,7 +29338,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$2:$C$12" spid="_x0000_s22557"/>
+                  <a14:cameraTool cellRange="$A$2:$C$12" spid="_x0000_s22559"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29402,7 +29402,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$2:$F$13" spid="_x0000_s7202"/>
+                  <a14:cameraTool cellRange="$B$2:$F$13" spid="_x0000_s7204"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29531,7 +29531,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$1:$F$24" spid="_x0000_s26679"/>
+                  <a14:cameraTool cellRange="$B$1:$F$24" spid="_x0000_s26683"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29595,7 +29595,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$26:$F$33" spid="_x0000_s26680"/>
+                  <a14:cameraTool cellRange="$B$26:$F$33" spid="_x0000_s26684"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29784,7 +29784,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$2:$F$10" spid="_x0000_s27715"/>
+                  <a14:cameraTool cellRange="$B$2:$F$10" spid="_x0000_s27719"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29848,7 +29848,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$12:$F$23" spid="_x0000_s27716"/>
+                  <a14:cameraTool cellRange="$B$12:$F$23" spid="_x0000_s27720"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30440,7 +30440,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$3:$G$11" spid="_x0000_s28781"/>
+                  <a14:cameraTool cellRange="$B$3:$G$11" spid="_x0000_s28789"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30504,7 +30504,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$13:$G$21" spid="_x0000_s28782"/>
+                  <a14:cameraTool cellRange="$B$13:$G$21" spid="_x0000_s28790"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30568,7 +30568,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$24:$G$29" spid="_x0000_s28783"/>
+                  <a14:cameraTool cellRange="$B$24:$G$29" spid="_x0000_s28791"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30632,7 +30632,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$31:$H$35" spid="_x0000_s28784"/>
+                  <a14:cameraTool cellRange="$B$31:$H$35" spid="_x0000_s28792"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30892,7 +30892,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$2:$F$14" spid="_x0000_s50183"/>
+                  <a14:cameraTool cellRange="$B$2:$F$14" spid="_x0000_s50185"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -31963,7 +31963,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$H$1:$L$20" spid="_x0000_s17471"/>
+                  <a14:cameraTool cellRange="$H$1:$L$20" spid="_x0000_s17475"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32010,7 +32010,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>13</xdr:col>
-          <xdr:colOff>38100</xdr:colOff>
+          <xdr:colOff>50800</xdr:colOff>
           <xdr:row>57</xdr:row>
           <xdr:rowOff>57150</xdr:rowOff>
         </xdr:to>
@@ -32027,7 +32027,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$A$1:$F$12" spid="_x0000_s17472"/>
+                  <a14:cameraTool cellRange="$A$1:$F$12" spid="_x0000_s17476"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32041,8 +32041,8 @@
           </xdr:blipFill>
           <xdr:spPr bwMode="auto">
             <a:xfrm>
-              <a:off x="4943475" y="7010400"/>
-              <a:ext cx="3771900" cy="1924050"/>
+              <a:off x="4933950" y="7010400"/>
+              <a:ext cx="3765550" cy="1924050"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -32134,7 +32134,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$59:$H$66" spid="_x0000_s14368"/>
+                  <a14:cameraTool cellRange="$B$59:$H$66" spid="_x0000_s14370"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32334,7 +32334,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$I$1:$N$14" spid="_x0000_s6178"/>
+                  <a14:cameraTool cellRange="$I$1:$N$14" spid="_x0000_s6180"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32441,7 +32441,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$3:$M$12" spid="_x0000_s10307"/>
+                  <a14:cameraTool cellRange="$B$3:$M$12" spid="_x0000_s10311"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32505,7 +32505,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$O$3:$S$8" spid="_x0000_s10308"/>
+                  <a14:cameraTool cellRange="$O$3:$S$8" spid="_x0000_s10312"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32634,7 +32634,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$3:$E$19" spid="_x0000_s11364"/>
+                  <a14:cameraTool cellRange="$B$3:$E$19" spid="_x0000_s11370"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32698,7 +32698,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$22:$E$28" spid="_x0000_s11365"/>
+                  <a14:cameraTool cellRange="$B$22:$E$28" spid="_x0000_s11371"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32762,7 +32762,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$B$31:$E$52" spid="_x0000_s11366"/>
+                  <a14:cameraTool cellRange="$B$31:$E$52" spid="_x0000_s11372"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -32847,9 +32847,6 @@
 <file path=xl/externalLinks/externalLink10.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:relativeUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="_TM_정리"/>
       <sheetName val="FS"/>
@@ -33661,9 +33658,6 @@
 <file path=xl/externalLinks/externalLink12.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:relativeUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="_TM_정리"/>
       <sheetName val="Assign"/>
@@ -34477,9 +34471,6 @@
 <file path=xl/externalLinks/externalLink9.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:relativeUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="_TM_정리"/>
       <sheetName val="overview"/>
@@ -34936,7 +34927,7 @@
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="16384" width="9" style="444"/>
   </cols>
@@ -34952,11 +34943,11 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="B3:E52"/>
-  <sheetFormatPr defaultRowHeight="19.5" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9" style="388"/>
-    <col min="2" max="2" width="18.375" style="388" customWidth="1"/>
-    <col min="3" max="5" width="9.625" style="388" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" style="388" customWidth="1"/>
+    <col min="3" max="5" width="9.58203125" style="388" customWidth="1"/>
     <col min="6" max="7" width="10.5" style="388" customWidth="1"/>
     <col min="8" max="16384" width="9" style="388"/>
   </cols>
@@ -35644,11 +35635,11 @@
     <tabColor rgb="FFFF9999"/>
   </sheetPr>
   <dimension ref="A1:J65"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="16.625" style="5" customWidth="1"/>
-    <col min="2" max="5" width="7.625" style="5" customWidth="1"/>
-    <col min="6" max="9" width="5.625" style="236" customWidth="1"/>
+    <col min="1" max="1" width="16.58203125" style="5" customWidth="1"/>
+    <col min="2" max="5" width="7.58203125" style="5" customWidth="1"/>
+    <col min="6" max="9" width="5.58203125" style="236" customWidth="1"/>
     <col min="10" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -37173,13 +37164,13 @@
     <tabColor rgb="FFFF9999"/>
   </sheetPr>
   <dimension ref="B2:I32"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="2.625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="12.625" style="5" customWidth="1"/>
-    <col min="3" max="4" width="8.625" style="5" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="8" width="8.625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="8.625" style="5" customWidth="1" outlineLevel="1"/>
+    <col min="1" max="1" width="2.58203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.58203125" style="5" customWidth="1"/>
+    <col min="3" max="4" width="8.58203125" style="5" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="8" width="8.58203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="8.58203125" style="5" customWidth="1" outlineLevel="1"/>
     <col min="10" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -37948,12 +37939,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="B1:F31"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9" style="388"/>
-    <col min="2" max="2" width="14.875" style="388" customWidth="1"/>
-    <col min="3" max="6" width="8.125" style="388" customWidth="1"/>
-    <col min="7" max="7" width="10.625" style="388" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" style="388" customWidth="1"/>
+    <col min="3" max="6" width="8.08203125" style="388" customWidth="1"/>
+    <col min="7" max="7" width="10.58203125" style="388" customWidth="1"/>
     <col min="8" max="16384" width="9" style="388"/>
   </cols>
   <sheetData>
@@ -38542,12 +38533,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="B1:G23"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9" style="388"/>
-    <col min="2" max="2" width="16.875" style="388" customWidth="1"/>
-    <col min="3" max="6" width="7.625" style="388" customWidth="1"/>
-    <col min="7" max="7" width="10.625" style="388" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" style="388" customWidth="1"/>
+    <col min="3" max="6" width="7.58203125" style="388" customWidth="1"/>
+    <col min="7" max="7" width="10.58203125" style="388" customWidth="1"/>
     <col min="8" max="16384" width="9" style="388"/>
   </cols>
   <sheetData>
@@ -38945,7 +38936,7 @@
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="17"/>
   <sheetData/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -38958,14 +38949,14 @@
     <tabColor rgb="FFFF9999"/>
   </sheetPr>
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="5.875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.58203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="5.83203125" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="8.75" style="5" customWidth="1"/>
-    <col min="7" max="7" width="8.625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="12.625" style="5" customWidth="1"/>
-    <col min="9" max="14" width="8.625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="8.58203125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.58203125" style="5" customWidth="1"/>
+    <col min="9" max="14" width="8.58203125" style="5" customWidth="1"/>
     <col min="15" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -39163,10 +39154,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="B1:F21"/>
-  <sheetFormatPr defaultRowHeight="12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9" style="591"/>
-    <col min="2" max="2" width="13.375" style="591" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" style="591" customWidth="1"/>
     <col min="3" max="6" width="8.25" style="591" customWidth="1"/>
     <col min="7" max="16384" width="9" style="591"/>
   </cols>
@@ -39468,7 +39459,7 @@
         <v>6169000000</v>
       </c>
     </row>
-    <row r="20" spans="2:6" ht="12.75" thickBot="1">
+    <row r="20" spans="2:6" ht="15" thickBot="1">
       <c r="B20" s="622" t="s">
         <v>134</v>
       </c>
@@ -39504,11 +39495,11 @@
     <tabColor rgb="FFFF9999"/>
   </sheetPr>
   <dimension ref="A1:J103"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="16.625" style="5" customWidth="1"/>
-    <col min="2" max="5" width="7.625" style="5" customWidth="1"/>
-    <col min="6" max="9" width="5.625" style="236" customWidth="1"/>
+    <col min="1" max="1" width="16.58203125" style="5" customWidth="1"/>
+    <col min="2" max="5" width="7.58203125" style="5" customWidth="1"/>
+    <col min="6" max="9" width="5.58203125" style="236" customWidth="1"/>
     <col min="10" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -41278,11 +41269,11 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C54"/>
-  <sheetFormatPr defaultRowHeight="21.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="21.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17.75" style="632" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.375" style="633" customWidth="1"/>
-    <col min="3" max="3" width="48.375" style="633" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" style="633" customWidth="1"/>
+    <col min="3" max="3" width="48.33203125" style="633" customWidth="1"/>
     <col min="4" max="16384" width="9" style="628"/>
   </cols>
   <sheetData>
@@ -41298,7 +41289,7 @@
       <c r="B2" s="630"/>
       <c r="C2" s="631"/>
     </row>
-    <row r="3" spans="1:3" ht="22.5">
+    <row r="3" spans="1:3" ht="23">
       <c r="A3" s="751" t="s">
         <v>379</v>
       </c>
@@ -41309,7 +41300,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="22.5">
+    <row r="4" spans="1:3" ht="23">
       <c r="A4" s="754" t="s">
         <v>382</v>
       </c>
@@ -41320,7 +41311,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="22.5">
+    <row r="5" spans="1:3" ht="23">
       <c r="A5" s="757" t="s">
         <v>382</v>
       </c>
@@ -41331,7 +41322,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="22.5">
+    <row r="6" spans="1:3" ht="23">
       <c r="A6" s="757" t="s">
         <v>387</v>
       </c>
@@ -41342,7 +41333,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="22.5">
+    <row r="7" spans="1:3" ht="23">
       <c r="A7" s="757" t="s">
         <v>387</v>
       </c>
@@ -41353,7 +41344,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="22.5">
+    <row r="8" spans="1:3" ht="23">
       <c r="A8" s="757" t="s">
         <v>387</v>
       </c>
@@ -41364,7 +41355,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="33.75">
+    <row r="9" spans="1:3" ht="34.5">
       <c r="A9" s="757" t="s">
         <v>394</v>
       </c>
@@ -41375,7 +41366,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="33.75">
+    <row r="10" spans="1:3" ht="34.5">
       <c r="A10" s="757" t="s">
         <v>397</v>
       </c>
@@ -41386,7 +41377,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="33.75">
+    <row r="11" spans="1:3" ht="34.5">
       <c r="A11" s="757" t="s">
         <v>397</v>
       </c>
@@ -41397,7 +41388,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="33.75">
+    <row r="12" spans="1:3" ht="34.5">
       <c r="A12" s="760" t="s">
         <v>397</v>
       </c>
@@ -41408,19 +41399,19 @@
         <v>403</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="11.25">
+    <row r="13" spans="1:3" ht="11.5">
       <c r="C13" s="634"/>
     </row>
-    <row r="14" spans="1:3" ht="11.25">
+    <row r="14" spans="1:3" ht="11.5">
       <c r="C14" s="634"/>
     </row>
-    <row r="15" spans="1:3" ht="11.25">
+    <row r="15" spans="1:3" ht="11.5">
       <c r="C15" s="634"/>
     </row>
-    <row r="16" spans="1:3" ht="11.25">
+    <row r="16" spans="1:3" ht="11.5">
       <c r="C16" s="634"/>
     </row>
-    <row r="17" spans="3:3" ht="11.25">
+    <row r="17" spans="3:3" ht="11.5">
       <c r="C17" s="634"/>
     </row>
     <row r="18" spans="3:3" ht="21.75" customHeight="1">
@@ -41457,13 +41448,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:K29"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="17"/>
   <cols>
-    <col min="2" max="2" width="11.375" customWidth="1"/>
-    <col min="3" max="3" width="35.875" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
     <col min="6" max="6" width="9.25" customWidth="1"/>
     <col min="7" max="7" width="38" customWidth="1"/>
-    <col min="9" max="9" width="26.625" customWidth="1"/>
+    <col min="9" max="9" width="26.58203125" customWidth="1"/>
     <col min="10" max="11" width="10.25" customWidth="1"/>
   </cols>
   <sheetData>
@@ -41784,12 +41775,12 @@
     <tabColor rgb="FFFF9999"/>
   </sheetPr>
   <dimension ref="B2:K40"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="2.625" style="29" customWidth="1"/>
-    <col min="2" max="2" width="14.625" style="29" customWidth="1"/>
-    <col min="3" max="6" width="8.125" style="29" customWidth="1"/>
-    <col min="7" max="9" width="8.625" style="29" customWidth="1"/>
+    <col min="1" max="1" width="2.58203125" style="29" customWidth="1"/>
+    <col min="2" max="2" width="14.58203125" style="29" customWidth="1"/>
+    <col min="3" max="6" width="8.08203125" style="29" customWidth="1"/>
+    <col min="7" max="9" width="8.58203125" style="29" customWidth="1"/>
     <col min="10" max="16384" width="9" style="29"/>
   </cols>
   <sheetData>
@@ -42431,15 +42422,15 @@
     <tabColor rgb="FFFF9999"/>
   </sheetPr>
   <dimension ref="B1:K34"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="2.625" style="251" customWidth="1"/>
-    <col min="2" max="2" width="12.625" style="251" customWidth="1"/>
+    <col min="1" max="1" width="2.58203125" style="251" customWidth="1"/>
+    <col min="2" max="2" width="12.58203125" style="251" customWidth="1"/>
     <col min="3" max="3" width="9.25" style="251" customWidth="1" outlineLevel="1"/>
-    <col min="4" max="4" width="9.375" style="251" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="7" width="8.625" style="251" customWidth="1"/>
-    <col min="8" max="8" width="8.625" style="251" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="8.625" style="251" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" style="251" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="7" width="8.58203125" style="251" customWidth="1"/>
+    <col min="8" max="8" width="8.58203125" style="251" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="8.58203125" style="251" customWidth="1"/>
     <col min="10" max="16384" width="9" style="251"/>
   </cols>
   <sheetData>
@@ -43320,12 +43311,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="B1:F33"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9" style="388"/>
-    <col min="2" max="2" width="16.875" style="388" customWidth="1"/>
-    <col min="3" max="6" width="7.625" style="388" customWidth="1"/>
-    <col min="7" max="7" width="10.625" style="388" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" style="388" customWidth="1"/>
+    <col min="3" max="6" width="7.58203125" style="388" customWidth="1"/>
+    <col min="7" max="7" width="10.58203125" style="388" customWidth="1"/>
     <col min="8" max="16384" width="9" style="388"/>
   </cols>
   <sheetData>
@@ -43971,12 +43962,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="B2:F25"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9" style="388"/>
-    <col min="2" max="2" width="16.875" style="388" customWidth="1"/>
-    <col min="3" max="6" width="7.625" style="388" customWidth="1"/>
-    <col min="7" max="7" width="10.625" style="388" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" style="388" customWidth="1"/>
+    <col min="3" max="6" width="7.58203125" style="388" customWidth="1"/>
+    <col min="7" max="7" width="10.58203125" style="388" customWidth="1"/>
     <col min="8" max="16384" width="9" style="388"/>
   </cols>
   <sheetData>
@@ -44286,11 +44277,11 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="B3:H35"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="9" style="705"/>
-    <col min="2" max="2" width="14.625" style="705" customWidth="1"/>
-    <col min="3" max="3" width="15.875" style="705" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.58203125" style="705" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" style="705" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" style="705" bestFit="1" customWidth="1"/>
     <col min="5" max="8" width="11.5" style="705" customWidth="1"/>
     <col min="9" max="10" width="9" style="705"/>
@@ -44695,7 +44686,7 @@
       <c r="F28" s="847"/>
       <c r="G28" s="853"/>
     </row>
-    <row r="29" spans="2:8" ht="13.5" thickBot="1">
+    <row r="29" spans="2:8" ht="13" thickBot="1">
       <c r="B29" s="770" t="s">
         <v>151</v>
       </c>
@@ -44798,7 +44789,7 @@
         <v>-139246979.81999999</v>
       </c>
     </row>
-    <row r="35" spans="2:8" ht="13.5" thickBot="1">
+    <row r="35" spans="2:8" ht="13" thickBot="1">
       <c r="B35" s="720" t="s">
         <v>151</v>
       </c>
@@ -44839,11 +44830,11 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <dimension ref="B1:F14"/>
-  <sheetFormatPr defaultRowHeight="11.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5"/>
   <cols>
     <col min="1" max="1" width="9" style="811"/>
     <col min="2" max="2" width="17.5" style="811" customWidth="1"/>
-    <col min="3" max="6" width="7.375" style="811" customWidth="1"/>
+    <col min="3" max="6" width="7.33203125" style="811" customWidth="1"/>
     <col min="7" max="16384" width="9" style="811"/>
   </cols>
   <sheetData>
@@ -45081,15 +45072,15 @@
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
   <dimension ref="A2:T63"/>
-  <sheetFormatPr defaultRowHeight="11.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="10"/>
   <cols>
     <col min="1" max="2" width="4" style="636" customWidth="1"/>
-    <col min="3" max="3" width="14.875" style="636" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" style="636" customWidth="1"/>
     <col min="4" max="8" width="11.75" style="636" customWidth="1"/>
     <col min="9" max="9" width="9" style="636"/>
     <col min="10" max="10" width="22.5" style="636" customWidth="1"/>
-    <col min="11" max="14" width="12.375" style="636" customWidth="1"/>
-    <col min="15" max="15" width="14.625" style="636" customWidth="1"/>
+    <col min="11" max="14" width="12.33203125" style="636" customWidth="1"/>
+    <col min="15" max="15" width="14.58203125" style="636" customWidth="1"/>
     <col min="16" max="20" width="13.25" style="636" customWidth="1"/>
     <col min="21" max="16384" width="9" style="636"/>
   </cols>
@@ -45104,7 +45095,7 @@
       <c r="E3" s="637"/>
       <c r="F3" s="637"/>
     </row>
-    <row r="4" spans="3:15">
+    <row r="4" spans="3:15" ht="11.5">
       <c r="C4" s="638" t="s">
         <v>57</v>
       </c>
@@ -45237,7 +45228,7 @@
         <v>80750096785</v>
       </c>
     </row>
-    <row r="7" spans="3:15">
+    <row r="7" spans="3:15" ht="11.5">
       <c r="C7" s="642" t="s">
         <v>68</v>
       </c>
@@ -45332,7 +45323,7 @@
         <v>96044850738</v>
       </c>
     </row>
-    <row r="10" spans="3:15">
+    <row r="10" spans="3:15" ht="10.5">
       <c r="J10" s="638" t="s">
         <v>71</v>
       </c>
@@ -45401,7 +45392,7 @@
         <v>118989031133.66666</v>
       </c>
     </row>
-    <row r="13" spans="3:15">
+    <row r="13" spans="3:15" ht="11.5">
       <c r="C13" s="643" t="s">
         <v>72</v>
       </c>
@@ -45466,7 +45457,7 @@
         <v>4977175857</v>
       </c>
     </row>
-    <row r="16" spans="3:15">
+    <row r="16" spans="3:15" ht="11.5">
       <c r="C16" s="647" t="s">
         <v>76</v>
       </c>
@@ -45598,7 +45589,7 @@
       <c r="E38" s="648"/>
       <c r="F38" s="648"/>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" ht="11.5">
       <c r="A39" s="648"/>
       <c r="B39" s="650" t="s">
         <v>77</v>
@@ -45609,7 +45600,7 @@
       <c r="F39" s="652"/>
       <c r="G39" s="653"/>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" ht="11.5">
       <c r="A40" s="648"/>
       <c r="B40" s="654"/>
       <c r="C40" s="655" t="s">
@@ -45628,7 +45619,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" ht="11.5">
       <c r="A41" s="648"/>
       <c r="B41" s="659" t="s">
         <v>82</v>
@@ -45649,7 +45640,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" ht="11.5">
       <c r="A42" s="648"/>
       <c r="B42" s="664" t="s">
         <v>86</v>
@@ -45675,7 +45666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" ht="11.5">
       <c r="A43" s="648"/>
       <c r="B43" s="667" t="s">
         <v>87</v>
@@ -45696,7 +45687,7 @@
         <v>78023354330</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" ht="11.5">
       <c r="A44" s="648"/>
       <c r="B44" s="667" t="s">
         <v>88</v>
@@ -45717,7 +45708,7 @@
         <v>14951300913</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" ht="11.5">
       <c r="A45" s="648"/>
       <c r="B45" s="670" t="s">
         <v>89</v>
@@ -45772,15 +45763,15 @@
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
   <dimension ref="A2:T63"/>
-  <sheetFormatPr defaultRowHeight="11.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="10"/>
   <cols>
     <col min="1" max="2" width="4" style="636" customWidth="1"/>
-    <col min="3" max="3" width="14.875" style="636" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" style="636" customWidth="1"/>
     <col min="4" max="8" width="11.75" style="636" customWidth="1"/>
     <col min="9" max="9" width="9" style="636"/>
     <col min="10" max="10" width="22.5" style="636" customWidth="1"/>
-    <col min="11" max="14" width="12.375" style="636" customWidth="1"/>
-    <col min="15" max="15" width="14.625" style="636" customWidth="1"/>
+    <col min="11" max="14" width="12.33203125" style="636" customWidth="1"/>
+    <col min="15" max="15" width="14.58203125" style="636" customWidth="1"/>
     <col min="16" max="20" width="13.25" style="636" customWidth="1"/>
     <col min="21" max="16384" width="9" style="636"/>
   </cols>
@@ -45795,7 +45786,7 @@
       <c r="E3" s="637"/>
       <c r="F3" s="637"/>
     </row>
-    <row r="4" spans="3:15">
+    <row r="4" spans="3:15" ht="11.5">
       <c r="C4" s="638" t="s">
         <v>57</v>
       </c>
@@ -46012,7 +46003,7 @@
         <v>64272000000</v>
       </c>
     </row>
-    <row r="9" spans="3:15">
+    <row r="9" spans="3:15" ht="11.5">
       <c r="C9" s="642" t="s">
         <v>68</v>
       </c>
@@ -46129,7 +46120,7 @@
         <v>78474000000</v>
       </c>
     </row>
-    <row r="13" spans="3:15">
+    <row r="13" spans="3:15" ht="11.5">
       <c r="C13" s="643" t="s">
         <v>72</v>
       </c>
@@ -46166,7 +46157,7 @@
         <v>80533000000</v>
       </c>
     </row>
-    <row r="14" spans="3:15">
+    <row r="14" spans="3:15" ht="10.5">
       <c r="C14" s="642" t="s">
         <v>90</v>
       </c>
@@ -46320,7 +46311,7 @@
         <v>103431666666.66667</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" ht="11.5">
       <c r="C18" s="647" t="s">
         <v>76</v>
       </c>
@@ -46360,7 +46351,7 @@
         <v>103431666666.66667</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" spans="1:15" ht="10.5">
       <c r="C19" s="648"/>
       <c r="D19" s="648" t="b">
         <f>E9-D9=D18</f>
@@ -46483,7 +46474,7 @@
       <c r="E38" s="648"/>
       <c r="F38" s="648"/>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" ht="10.5">
       <c r="A39" s="648"/>
       <c r="B39" s="676" t="s">
         <v>94</v>
@@ -46494,7 +46485,7 @@
       <c r="F39" s="677"/>
       <c r="G39" s="678"/>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" ht="10.5">
       <c r="A40" s="648"/>
       <c r="B40" s="679" t="s">
         <v>95</v>
@@ -46513,7 +46504,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" ht="10.5">
       <c r="A41" s="648"/>
       <c r="B41" s="683"/>
       <c r="C41" s="684"/>
@@ -46608,7 +46599,7 @@
         <v>6169000000</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" ht="10.5">
       <c r="A46" s="648"/>
       <c r="B46" s="691"/>
       <c r="C46" s="694" t="s">
@@ -46667,7 +46658,7 @@
         <v>1569000000</v>
       </c>
     </row>
-    <row r="49" spans="2:20">
+    <row r="49" spans="2:20" ht="10.5">
       <c r="B49" s="691"/>
       <c r="C49" s="694" t="s">
         <v>102</v>
@@ -46685,7 +46676,7 @@
         <v>14296000000</v>
       </c>
     </row>
-    <row r="50" spans="2:20" ht="12" thickBot="1">
+    <row r="50" spans="2:20" ht="11" thickBot="1">
       <c r="B50" s="697"/>
       <c r="C50" s="698" t="s">
         <v>103</v>
@@ -46728,17 +46719,17 @@
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
   <dimension ref="A2:T63"/>
-  <sheetFormatPr defaultRowHeight="11.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="10"/>
   <cols>
     <col min="1" max="2" width="4" style="636" customWidth="1"/>
-    <col min="3" max="3" width="14.875" style="636" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" style="636" customWidth="1"/>
     <col min="4" max="6" width="11.75" style="636" customWidth="1"/>
-    <col min="7" max="7" width="13.125" style="636" customWidth="1"/>
+    <col min="7" max="7" width="13.08203125" style="636" customWidth="1"/>
     <col min="8" max="8" width="11.75" style="636" customWidth="1"/>
     <col min="9" max="9" width="13.75" style="636" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.5" style="636" customWidth="1"/>
-    <col min="11" max="14" width="12.375" style="636" customWidth="1"/>
-    <col min="15" max="15" width="14.625" style="636" customWidth="1"/>
+    <col min="11" max="14" width="12.33203125" style="636" customWidth="1"/>
+    <col min="15" max="15" width="14.58203125" style="636" customWidth="1"/>
     <col min="16" max="20" width="13.25" style="636" customWidth="1"/>
     <col min="21" max="16384" width="9" style="636"/>
   </cols>
@@ -46753,7 +46744,7 @@
       <c r="E3" s="637"/>
       <c r="F3" s="637"/>
     </row>
-    <row r="4" spans="3:15">
+    <row r="4" spans="3:15" ht="11.5">
       <c r="C4" s="638" t="s">
         <v>57</v>
       </c>
@@ -46886,7 +46877,7 @@
         <v>17617000000</v>
       </c>
     </row>
-    <row r="7" spans="3:15">
+    <row r="7" spans="3:15" ht="11.5">
       <c r="C7" s="642" t="s">
         <v>68</v>
       </c>
@@ -46985,7 +46976,7 @@
         <v>14958000000</v>
       </c>
     </row>
-    <row r="10" spans="3:15">
+    <row r="10" spans="3:15" ht="10.5">
       <c r="J10" s="638" t="s">
         <v>71</v>
       </c>
@@ -47054,7 +47045,7 @@
         <v>18482333333.333336</v>
       </c>
     </row>
-    <row r="13" spans="3:15">
+    <row r="13" spans="3:15" ht="11.5">
       <c r="C13" s="643" t="s">
         <v>72</v>
       </c>
@@ -47119,7 +47110,7 @@
         <v>579000000</v>
       </c>
     </row>
-    <row r="16" spans="3:15">
+    <row r="16" spans="3:15" ht="11.5">
       <c r="C16" s="647" t="s">
         <v>76</v>
       </c>
@@ -47251,7 +47242,7 @@
       <c r="E38" s="648"/>
       <c r="F38" s="648"/>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" ht="11.5">
       <c r="A39" s="648"/>
       <c r="B39" s="676" t="s">
         <v>104</v>
@@ -47262,7 +47253,7 @@
       <c r="F39" s="677"/>
       <c r="G39" s="678"/>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" ht="11.5">
       <c r="A40" s="648"/>
       <c r="B40" s="679" t="s">
         <v>105</v>
@@ -47281,7 +47272,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" ht="11.5">
       <c r="A41" s="648"/>
       <c r="B41" s="683"/>
       <c r="C41" s="684"/>
@@ -47298,7 +47289,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" ht="11.5">
       <c r="A42" s="648"/>
       <c r="B42" s="687" t="s">
         <v>111</v>
@@ -47319,7 +47310,7 @@
         <v>12727000000</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" ht="11.5">
       <c r="A43" s="648"/>
       <c r="B43" s="691"/>
       <c r="C43" s="636" t="s">
@@ -47338,7 +47329,7 @@
         <v>1569000000</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" ht="11.5">
       <c r="A44" s="648"/>
       <c r="B44" s="691"/>
       <c r="C44" s="694" t="s">
@@ -47410,14 +47401,14 @@
     <tabColor rgb="FFFF9999"/>
   </sheetPr>
   <dimension ref="A1:N37"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="8.625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="5.875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.58203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="5.83203125" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="8.75" style="5" customWidth="1"/>
-    <col min="7" max="7" width="8.625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="12.625" style="5" customWidth="1"/>
-    <col min="9" max="14" width="8.625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="8.58203125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="12.58203125" style="5" customWidth="1"/>
+    <col min="9" max="14" width="8.58203125" style="5" customWidth="1"/>
     <col min="15" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -48409,13 +48400,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B5:H66"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9" style="29"/>
-    <col min="2" max="2" width="8.625" style="29" customWidth="1"/>
-    <col min="3" max="3" width="9.625" style="29" customWidth="1"/>
-    <col min="4" max="7" width="7.125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="8.625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="8.58203125" style="29" customWidth="1"/>
+    <col min="3" max="3" width="9.58203125" style="29" customWidth="1"/>
+    <col min="4" max="7" width="7.08203125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="8.58203125" style="29" customWidth="1"/>
     <col min="9" max="16384" width="9" style="29"/>
   </cols>
   <sheetData>
@@ -49276,15 +49267,15 @@
     <tabColor rgb="FFFF9999"/>
   </sheetPr>
   <dimension ref="B1:N38"/>
-  <sheetFormatPr defaultRowHeight="12" customHeight="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" customHeight="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="2.625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="12.625" style="5" customWidth="1"/>
-    <col min="3" max="5" width="8.625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="8.625" style="5" customWidth="1" outlineLevel="1"/>
-    <col min="7" max="8" width="8.625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="12.625" style="5" customWidth="1"/>
-    <col min="10" max="16" width="8.625" style="5" customWidth="1"/>
+    <col min="1" max="1" width="2.58203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.58203125" style="5" customWidth="1"/>
+    <col min="3" max="5" width="8.58203125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="8.58203125" style="5" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="8" width="8.58203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="12.58203125" style="5" customWidth="1"/>
+    <col min="10" max="16" width="8.58203125" style="5" customWidth="1"/>
     <col min="17" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -50484,24 +50475,24 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="B3:S13"/>
-  <sheetFormatPr defaultRowHeight="11.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5"/>
   <cols>
     <col min="1" max="1" width="5.75" style="251" customWidth="1"/>
-    <col min="2" max="2" width="5.125" style="251" customWidth="1"/>
-    <col min="3" max="3" width="7.125" style="251" customWidth="1"/>
-    <col min="4" max="4" width="4.375" style="385" customWidth="1"/>
-    <col min="5" max="5" width="5.125" style="251" customWidth="1"/>
-    <col min="6" max="6" width="7.125" style="251" customWidth="1"/>
-    <col min="7" max="7" width="4.375" style="385" customWidth="1"/>
-    <col min="8" max="8" width="5.125" style="251" customWidth="1"/>
-    <col min="9" max="9" width="7.125" style="251" customWidth="1"/>
-    <col min="10" max="10" width="4.375" style="385" customWidth="1"/>
-    <col min="11" max="11" width="5.125" style="251" customWidth="1"/>
-    <col min="12" max="12" width="7.125" style="251" customWidth="1"/>
-    <col min="13" max="13" width="4.375" style="385" customWidth="1"/>
+    <col min="2" max="2" width="5.08203125" style="251" customWidth="1"/>
+    <col min="3" max="3" width="7.08203125" style="251" customWidth="1"/>
+    <col min="4" max="4" width="4.33203125" style="385" customWidth="1"/>
+    <col min="5" max="5" width="5.08203125" style="251" customWidth="1"/>
+    <col min="6" max="6" width="7.08203125" style="251" customWidth="1"/>
+    <col min="7" max="7" width="4.33203125" style="385" customWidth="1"/>
+    <col min="8" max="8" width="5.08203125" style="251" customWidth="1"/>
+    <col min="9" max="9" width="7.08203125" style="251" customWidth="1"/>
+    <col min="10" max="10" width="4.33203125" style="385" customWidth="1"/>
+    <col min="11" max="11" width="5.08203125" style="251" customWidth="1"/>
+    <col min="12" max="12" width="7.08203125" style="251" customWidth="1"/>
+    <col min="13" max="13" width="4.33203125" style="385" customWidth="1"/>
     <col min="14" max="14" width="9" style="251"/>
-    <col min="15" max="15" width="14.875" style="251" customWidth="1"/>
-    <col min="16" max="19" width="6.125" style="251" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" style="251" customWidth="1"/>
+    <col min="16" max="19" width="6.08203125" style="251" customWidth="1"/>
     <col min="20" max="16384" width="9" style="251"/>
   </cols>
   <sheetData>

</xml_diff>